<commit_message>
fix(parser): silently coerce int/float/bool cells to string in pattern files
Excel auto-types cells typed without a leading apostrophe. Rejecting them
produced a confusing SecurityError for common cases like typing 1 for
pattern.version.

Changes:
- int, float (whole number, no decimal), bool: coerced to str silently
- datetime/date/time: still rejected (ambiguous in a pattern context)
- Formulas: still rejected (security)

Tests updated: numeric/boolean rejected tests become coerced tests;
new datetime-rejected tests added in both test files.
Snapshot for 03_purchase_order manual regenerated (pattern.version now
explicitly declared, stored as integer 1 by Excel, coerced to string).

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01K6EyxWBecbqyp9uRx7c4J8
</commit_message>
<xml_diff>
--- a/tests/fixtures/03_purchase_order/03_purchase_order_pattern-manual.xlsx
+++ b/tests/fixtures/03_purchase_order/03_purchase_order_pattern-manual.xlsx
@@ -20,9 +20,12 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="120" uniqueCount="55">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="122" uniqueCount="56">
   <si>
     <t xml:space="preserve">config:</t>
+  </si>
+  <si>
+    <t xml:space="preserve">pattern.version</t>
   </si>
   <si>
     <t xml:space="preserve">read.direction</t>
@@ -577,7 +580,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:G1048576"/>
+  <dimension ref="A1:G37"/>
   <sheetFormatPr defaultColWidth="10.16015625" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="7.51"/>
@@ -590,29 +593,25 @@
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="1" t="s">
+      <c r="A1" s="0" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" s="0" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="1" t="s">
-        <v>2</v>
-      </c>
-      <c r="D1" s="1"/>
-      <c r="E1" s="1"/>
-      <c r="F1" s="1"/>
-      <c r="G1" s="1"/>
+      <c r="C1" s="0" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="1" t="s">
         <v>0</v>
       </c>
       <c r="B2" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="C2" s="1" t="s">
         <v>3</v>
-      </c>
-      <c r="C2" s="1" t="s">
-        <v>4</v>
       </c>
       <c r="D2" s="1"/>
       <c r="E2" s="1"/>
@@ -620,34 +619,32 @@
       <c r="G2" s="1"/>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="2" t="s">
+      <c r="A3" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B3" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="C3" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="B3" s="2" t="s">
-        <v>6</v>
-      </c>
-      <c r="C3" s="2" t="s">
-        <v>7</v>
-      </c>
-      <c r="D3" s="2" t="s">
-        <v>8</v>
-      </c>
-      <c r="E3" s="2"/>
-      <c r="F3" s="2"/>
-      <c r="G3" s="2"/>
+      <c r="D3" s="1"/>
+      <c r="E3" s="1"/>
+      <c r="F3" s="1"/>
+      <c r="G3" s="1"/>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="2" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="B4" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="C4" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="D4" s="2" t="s">
         <v>9</v>
-      </c>
-      <c r="C4" s="2" t="s">
-        <v>7</v>
-      </c>
-      <c r="D4" s="2" t="s">
-        <v>10</v>
       </c>
       <c r="E4" s="2"/>
       <c r="F4" s="2"/>
@@ -655,16 +652,16 @@
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="2" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="B5" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="C5" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="D5" s="2" t="s">
         <v>11</v>
-      </c>
-      <c r="C5" s="2" t="s">
-        <v>7</v>
-      </c>
-      <c r="D5" s="2" t="s">
-        <v>12</v>
       </c>
       <c r="E5" s="2"/>
       <c r="F5" s="2"/>
@@ -672,16 +669,16 @@
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="2" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="B6" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="C6" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="D6" s="2" t="s">
         <v>13</v>
-      </c>
-      <c r="C6" s="2" t="s">
-        <v>7</v>
-      </c>
-      <c r="D6" s="2" t="s">
-        <v>14</v>
       </c>
       <c r="E6" s="2"/>
       <c r="F6" s="2"/>
@@ -689,16 +686,16 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="2" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="B7" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="C7" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="D7" s="2" t="s">
         <v>15</v>
-      </c>
-      <c r="C7" s="2" t="s">
-        <v>7</v>
-      </c>
-      <c r="D7" s="2" t="s">
-        <v>16</v>
       </c>
       <c r="E7" s="2"/>
       <c r="F7" s="2"/>
@@ -706,16 +703,16 @@
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="2" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="B8" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="C8" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="D8" s="2" t="s">
         <v>17</v>
-      </c>
-      <c r="C8" s="2" t="s">
-        <v>7</v>
-      </c>
-      <c r="D8" s="2" t="s">
-        <v>18</v>
       </c>
       <c r="E8" s="2"/>
       <c r="F8" s="2"/>
@@ -723,16 +720,16 @@
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="2" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="B9" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="C9" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="D9" s="2" t="s">
         <v>19</v>
-      </c>
-      <c r="C9" s="2" t="s">
-        <v>7</v>
-      </c>
-      <c r="D9" s="2" t="s">
-        <v>20</v>
       </c>
       <c r="E9" s="2"/>
       <c r="F9" s="2"/>
@@ -740,16 +737,16 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="2" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="B10" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="C10" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="D10" s="2" t="s">
         <v>21</v>
-      </c>
-      <c r="C10" s="2" t="s">
-        <v>7</v>
-      </c>
-      <c r="D10" s="2" t="s">
-        <v>22</v>
       </c>
       <c r="E10" s="2"/>
       <c r="F10" s="2"/>
@@ -757,16 +754,16 @@
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="2" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="B11" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="C11" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="D11" s="2" t="s">
         <v>23</v>
-      </c>
-      <c r="C11" s="2" t="s">
-        <v>7</v>
-      </c>
-      <c r="D11" s="2" t="s">
-        <v>24</v>
       </c>
       <c r="E11" s="2"/>
       <c r="F11" s="2"/>
@@ -774,82 +771,82 @@
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="2" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="B12" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="C12" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="D12" s="2" t="s">
         <v>25</v>
-      </c>
-      <c r="C12" s="2" t="s">
-        <v>7</v>
-      </c>
-      <c r="D12" s="2" t="s">
-        <v>26</v>
       </c>
       <c r="E12" s="2"/>
       <c r="F12" s="2"/>
       <c r="G12" s="2"/>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A13" s="3" t="s">
+      <c r="A13" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="B13" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="C13" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="D13" s="2" t="s">
         <v>27</v>
       </c>
-      <c r="B13" s="3" t="s">
-        <v>28</v>
-      </c>
-      <c r="C13" s="3" t="s">
-        <v>7</v>
-      </c>
-      <c r="D13" s="3" t="s">
-        <v>29</v>
-      </c>
-      <c r="E13" s="3"/>
-      <c r="F13" s="3"/>
-      <c r="G13" s="3"/>
+      <c r="E13" s="2"/>
+      <c r="F13" s="2"/>
+      <c r="G13" s="2"/>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="3" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="B14" s="3" t="s">
+        <v>29</v>
+      </c>
+      <c r="C14" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="D14" s="3" t="s">
         <v>30</v>
       </c>
-      <c r="C14" s="3" t="s">
-        <v>31</v>
-      </c>
-      <c r="D14" s="3"/>
       <c r="E14" s="3"/>
       <c r="F14" s="3"/>
       <c r="G14" s="3"/>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="3" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="B15" s="3" t="s">
+        <v>31</v>
+      </c>
+      <c r="C15" s="3" t="s">
         <v>32</v>
       </c>
-      <c r="C15" s="3" t="s">
-        <v>7</v>
-      </c>
-      <c r="D15" s="3" t="s">
-        <v>33</v>
-      </c>
+      <c r="D15" s="3"/>
       <c r="E15" s="3"/>
       <c r="F15" s="3"/>
       <c r="G15" s="3"/>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="3" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="B16" s="3" t="s">
+        <v>33</v>
+      </c>
+      <c r="C16" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="D16" s="3" t="s">
         <v>34</v>
-      </c>
-      <c r="C16" s="3" t="s">
-        <v>7</v>
-      </c>
-      <c r="D16" s="3" t="s">
-        <v>35</v>
       </c>
       <c r="E16" s="3"/>
       <c r="F16" s="3"/>
@@ -857,16 +854,16 @@
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="3" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="B17" s="3" t="s">
+        <v>35</v>
+      </c>
+      <c r="C17" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="D17" s="3" t="s">
         <v>36</v>
-      </c>
-      <c r="C17" s="3" t="s">
-        <v>7</v>
-      </c>
-      <c r="D17" s="3" t="s">
-        <v>33</v>
       </c>
       <c r="E17" s="3"/>
       <c r="F17" s="3"/>
@@ -874,16 +871,16 @@
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="3" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="B18" s="3" t="s">
         <v>37</v>
       </c>
       <c r="C18" s="3" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="D18" s="3" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="E18" s="3"/>
       <c r="F18" s="3"/>
@@ -891,16 +888,16 @@
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="3" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="B19" s="3" t="s">
         <v>38</v>
       </c>
       <c r="C19" s="3" t="s">
-        <v>39</v>
+        <v>8</v>
       </c>
       <c r="D19" s="3" t="s">
-        <v>40</v>
+        <v>34</v>
       </c>
       <c r="E19" s="3"/>
       <c r="F19" s="3"/>
@@ -908,28 +905,30 @@
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="3" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="B20" s="3" t="s">
+        <v>39</v>
+      </c>
+      <c r="C20" s="3" t="s">
+        <v>40</v>
+      </c>
+      <c r="D20" s="3" t="s">
         <v>41</v>
       </c>
-      <c r="C20" s="3" t="s">
-        <v>42</v>
-      </c>
-      <c r="D20" s="3"/>
       <c r="E20" s="3"/>
       <c r="F20" s="3"/>
       <c r="G20" s="3"/>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="3" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="B21" s="3" t="s">
+        <v>42</v>
+      </c>
+      <c r="C21" s="3" t="s">
         <v>43</v>
-      </c>
-      <c r="C21" s="3" t="s">
-        <v>42</v>
       </c>
       <c r="D21" s="3"/>
       <c r="E21" s="3"/>
@@ -938,51 +937,53 @@
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="3" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="B22" s="3" t="s">
         <v>44</v>
       </c>
       <c r="C22" s="3" t="s">
-        <v>42</v>
-      </c>
-      <c r="D22" s="3" t="s">
-        <v>45</v>
-      </c>
+        <v>43</v>
+      </c>
+      <c r="D22" s="3"/>
       <c r="E22" s="3"/>
       <c r="F22" s="3"/>
       <c r="G22" s="3"/>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A23" s="4" t="s">
+      <c r="A23" s="3" t="s">
+        <v>28</v>
+      </c>
+      <c r="B23" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="C23" s="3" t="s">
+        <v>43</v>
+      </c>
+      <c r="D23" s="3" t="s">
         <v>46</v>
       </c>
-      <c r="B23" s="4"/>
-      <c r="C23" s="4"/>
-      <c r="D23" s="4"/>
-      <c r="E23" s="4"/>
-      <c r="F23" s="4"/>
-      <c r="G23" s="4"/>
+      <c r="E23" s="3"/>
+      <c r="F23" s="3"/>
+      <c r="G23" s="3"/>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A24" s="5" t="s">
+      <c r="A24" s="4" t="s">
         <v>47</v>
       </c>
-      <c r="B24" s="2" t="s">
-        <v>6</v>
-      </c>
-      <c r="C24" s="5"/>
-      <c r="D24" s="5"/>
-      <c r="E24" s="5"/>
-      <c r="F24" s="5"/>
-      <c r="G24" s="5"/>
+      <c r="B24" s="4"/>
+      <c r="C24" s="4"/>
+      <c r="D24" s="4"/>
+      <c r="E24" s="4"/>
+      <c r="F24" s="4"/>
+      <c r="G24" s="4"/>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="5" t="s">
         <v>48</v>
       </c>
-      <c r="B25" s="3" t="s">
-        <v>28</v>
+      <c r="B25" s="2" t="s">
+        <v>7</v>
       </c>
       <c r="C25" s="5"/>
       <c r="D25" s="5"/>
@@ -992,10 +993,10 @@
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="5" t="s">
-        <v>48</v>
-      </c>
-      <c r="B26" s="2" t="s">
-        <v>9</v>
+        <v>49</v>
+      </c>
+      <c r="B26" s="3" t="s">
+        <v>29</v>
       </c>
       <c r="C26" s="5"/>
       <c r="D26" s="5"/>
@@ -1005,10 +1006,10 @@
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="5" t="s">
-        <v>48</v>
-      </c>
-      <c r="B27" s="3" t="s">
-        <v>30</v>
+        <v>49</v>
+      </c>
+      <c r="B27" s="2" t="s">
+        <v>10</v>
       </c>
       <c r="C27" s="5"/>
       <c r="D27" s="5"/>
@@ -1018,10 +1019,10 @@
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="5" t="s">
-        <v>48</v>
-      </c>
-      <c r="B28" s="2" t="s">
-        <v>11</v>
+        <v>49</v>
+      </c>
+      <c r="B28" s="3" t="s">
+        <v>31</v>
       </c>
       <c r="C28" s="5"/>
       <c r="D28" s="5"/>
@@ -1031,10 +1032,10 @@
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="5" t="s">
-        <v>48</v>
-      </c>
-      <c r="B29" s="3" t="s">
-        <v>32</v>
+        <v>49</v>
+      </c>
+      <c r="B29" s="2" t="s">
+        <v>12</v>
       </c>
       <c r="C29" s="5"/>
       <c r="D29" s="5"/>
@@ -1044,10 +1045,10 @@
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="5" t="s">
-        <v>48</v>
-      </c>
-      <c r="B30" s="2" t="s">
-        <v>13</v>
+        <v>49</v>
+      </c>
+      <c r="B30" s="3" t="s">
+        <v>33</v>
       </c>
       <c r="C30" s="5"/>
       <c r="D30" s="5"/>
@@ -1057,10 +1058,10 @@
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A31" s="5" t="s">
-        <v>48</v>
-      </c>
-      <c r="B31" s="3" t="s">
-        <v>34</v>
+        <v>49</v>
+      </c>
+      <c r="B31" s="2" t="s">
+        <v>14</v>
       </c>
       <c r="C31" s="5"/>
       <c r="D31" s="5"/>
@@ -1069,91 +1070,103 @@
       <c r="G31" s="5"/>
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A32" s="6" t="s">
+      <c r="A32" s="5" t="s">
         <v>49</v>
       </c>
-      <c r="B32" s="6"/>
-      <c r="C32" s="6"/>
-      <c r="D32" s="6"/>
-      <c r="E32" s="6"/>
-      <c r="F32" s="6"/>
-      <c r="G32" s="6"/>
+      <c r="B32" s="3" t="s">
+        <v>35</v>
+      </c>
+      <c r="C32" s="5"/>
+      <c r="D32" s="5"/>
+      <c r="E32" s="5"/>
+      <c r="F32" s="5"/>
+      <c r="G32" s="5"/>
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A33" s="2"/>
-      <c r="B33" s="2" t="s">
+      <c r="A33" s="6" t="s">
         <v>50</v>
       </c>
-      <c r="C33" s="2" t="s">
-        <v>15</v>
-      </c>
-      <c r="D33" s="2" t="s">
-        <v>17</v>
-      </c>
-      <c r="E33" s="2" t="s">
-        <v>19</v>
-      </c>
-      <c r="F33" s="2" t="s">
-        <v>21</v>
-      </c>
-      <c r="G33" s="2" t="s">
-        <v>23</v>
-      </c>
+      <c r="B33" s="6"/>
+      <c r="C33" s="6"/>
+      <c r="D33" s="6"/>
+      <c r="E33" s="6"/>
+      <c r="F33" s="6"/>
+      <c r="G33" s="6"/>
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A34" s="3"/>
-      <c r="B34" s="3" t="s">
+      <c r="A34" s="2"/>
+      <c r="B34" s="2" t="s">
         <v>51</v>
       </c>
-      <c r="C34" s="3" t="s">
-        <v>36</v>
-      </c>
-      <c r="D34" s="3" t="s">
+      <c r="C34" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="D34" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="E34" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="F34" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="G34" s="2" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A35" s="3"/>
+      <c r="B35" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="C35" s="3" t="s">
         <v>37</v>
       </c>
-      <c r="E34" s="3" t="s">
+      <c r="D35" s="3" t="s">
         <v>38</v>
       </c>
-      <c r="F34" s="3" t="s">
-        <v>41</v>
-      </c>
-      <c r="G34" s="3" t="s">
-        <v>43</v>
-      </c>
-    </row>
-    <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A35" s="1"/>
-      <c r="B35" s="1" t="s">
-        <v>52</v>
-      </c>
-      <c r="C35" s="2" t="s">
-        <v>25</v>
-      </c>
-      <c r="D35" s="1" t="s">
-        <v>53</v>
-      </c>
-      <c r="E35" s="1" t="s">
-        <v>53</v>
-      </c>
-      <c r="F35" s="1" t="s">
-        <v>53</v>
+      <c r="E35" s="3" t="s">
+        <v>39</v>
+      </c>
+      <c r="F35" s="3" t="s">
+        <v>42</v>
       </c>
       <c r="G35" s="3" t="s">
         <v>44</v>
       </c>
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A36" s="4" t="s">
+      <c r="A36" s="1"/>
+      <c r="B36" s="1" t="s">
+        <v>53</v>
+      </c>
+      <c r="C36" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="D36" s="1" t="s">
         <v>54</v>
       </c>
-      <c r="B36" s="4"/>
-      <c r="C36" s="4"/>
-      <c r="D36" s="4"/>
-      <c r="E36" s="4"/>
-      <c r="F36" s="4"/>
-      <c r="G36" s="4"/>
-    </row>
-    <row r="1048576" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+      <c r="E36" s="1" t="s">
+        <v>54</v>
+      </c>
+      <c r="F36" s="1" t="s">
+        <v>54</v>
+      </c>
+      <c r="G36" s="3" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A37" s="4" t="s">
+        <v>55</v>
+      </c>
+      <c r="B37" s="4"/>
+      <c r="C37" s="4"/>
+      <c r="D37" s="4"/>
+      <c r="E37" s="4"/>
+      <c r="F37" s="4"/>
+      <c r="G37" s="4"/>
+    </row>
   </sheetData>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>

</xml_diff>